<commit_message>
feat: adiciona campos de cidade e ordem nas lojas, ordena listagem e aprimora layout do StoreCard
</commit_message>
<xml_diff>
--- a/sodanca-latinamerica-import.xlsx
+++ b/sodanca-latinamerica-import.xlsx
@@ -552,391 +552,412 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K27"/>
+  <dimension ref="A1:M26"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
         <v>Nome</v>
       </c>
       <c r="B1" t="str">
+        <v>Cidade</v>
+      </c>
+      <c r="C1" t="str">
         <v>Slug</v>
       </c>
-      <c r="C1" t="str">
+      <c r="D1" t="str">
         <v>Pais (slug)</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
         <v>Endereco</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>LinkMaps</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>Telefone</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>Email</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>Instagram</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>Facebook</v>
       </c>
-      <c r="J1" t="str">
+      <c r="K1" t="str">
         <v>Website</v>
       </c>
-      <c r="K1" t="str">
+      <c r="L1" t="str">
         <v>Logo (arquivo)</v>
+      </c>
+      <c r="M1" t="str">
+        <v>Ordem</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>The Dance Shop</v>
+        <v>FOUETTE</v>
       </c>
       <c r="B2" t="str">
-        <v>the-dance-shop-montevideo-carrasco</v>
+        <v>Mendoza</v>
       </c>
       <c r="C2" t="str">
-        <v>uruguay</v>
+        <v>fouette-mendoza</v>
       </c>
       <c r="D2" t="str">
-        <v>Carlos Sáez y Arocena, Galeria Roma Local 1</v>
+        <v>argentina</v>
       </c>
       <c r="E2" t="str">
-        <v/>
+        <v>Lavalle 35/45 local 34 Galería Independencia - Mendoza Capital</v>
       </c>
       <c r="F2" t="str">
-        <v>+598 91 463 106</v>
+        <v>https://www.google.com/maps/place/Galer%C3%ADa+Independencia/@-32.8885556,-68.8380256,3a,75y,157.02h,91.78t/data=!3m7!1e1!3m5!1s8tSur1-aHdwxmAjLuXr1YA!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-1.7792920309981781%26panoid%3D8tSur1-aHdwxmAjLuXr1YA%26yaw%3D157.02122739013302!7i16384!8i8192!4m14!1m7!3m6!1s0x967e091906ac3fb5:0xd1f38edf52822e93!2sGaler%C3%ADa+Independencia!8m2!3d-32.8890198!4d-68.8381173!16s%2Fg%2F11bw4hy0dt!3m5!1s0x967e091906ac3fb5:0xd1f38edf52822e93!8m2!3d-32.8890198!4d-68.8381173!16s%2Fg%2F11bw4hy0dt?coh=205410&amp;entry=ttu&amp;g_ep=EgoyMDI0MTAwMi4xIKXMDSoASAFQAw%3D%3D</v>
       </c>
       <c r="G2" t="str">
-        <v>danceshop.uy@gmail.com</v>
+        <v>+54 911 5724-1569</v>
       </c>
       <c r="H2" t="str">
-        <v/>
+        <v>ventas@32fouette.com.ar</v>
       </c>
       <c r="I2" t="str">
-        <v/>
-      </c>
-      <c r="J2" t="str">
-        <v>https://thedanceshop.com.uy/</v>
+        <v>https://www.instagram.com/fouette.mendoza/</v>
       </c>
       <c r="K2" t="str">
-        <v>media-1333.jpg</v>
+        <v>https://fouette.com.ar/</v>
+      </c>
+      <c r="L2" t="str">
+        <v>7.jpg</v>
+      </c>
+      <c r="M2">
+        <v>1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>The Dance Shop</v>
+        <v>FOUETTE</v>
       </c>
       <c r="B3" t="str">
-        <v>the-dance-shop-montevideo-punta-carretas</v>
+        <v>Córdoba</v>
       </c>
       <c r="C3" t="str">
-        <v>uruguay</v>
+        <v>fouette-cordoba</v>
       </c>
       <c r="D3" t="str">
-        <v>21 de setiembre 2951, esq. Tomás Diago</v>
+        <v>argentina</v>
       </c>
       <c r="E3" t="str">
-        <v/>
+        <v>Córdoba 3068, Mar del Plata</v>
       </c>
       <c r="F3" t="str">
-        <v>+598 91 463 106</v>
+        <v>https://www.google.com/maps/place/Fouette/@-38.0103675,-57.5557138,3a,75y,115.85h,95.65t/data=!3m7!1e1!3m5!1srJ_sVXyToxFHfgHDvafsNw!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-5.65189321189014%26panoid%3DrJ_sVXyToxFHfgHDvafsNw%26yaw%3D115.85355644268819!7i16384!8i8192!4m16!1m9!3m8!1s0x9584dea049a0f1e5:0x723a3a938bbc32eb!2sC%C3%B3rdoba+3068,+B7602CAF+Mar+del+Plata,+Provincia+de+Buenos+Aires,+Argentina!3b1!8m2!3d-38.0104545!4d-57.5556471!10e5!16s%2Fg%2F11f3w1nnm1!3m5!1s0x9584dea049afa063:0x3d327ea0788c0499!8m2!3d-38.0104238!4d-57.5556416!16s%2Fg%2F11bwf7fsp0?coh=205410&amp;entry=ttu&amp;g_ep=EgoyMDI0MTAwMi4xIKXMDSoASAFQAw%3D%3D</v>
       </c>
       <c r="G3" t="str">
-        <v>danceshop.uy@gmail.com</v>
+        <v>+54 911 5723-6341</v>
       </c>
       <c r="H3" t="str">
-        <v/>
+        <v>ventas@32fouette.com.ar</v>
       </c>
       <c r="I3" t="str">
-        <v/>
-      </c>
-      <c r="J3" t="str">
-        <v>https://thedanceshop.com.uy/</v>
+        <v>https://www.instagram.com/fouette_32</v>
       </c>
       <c r="K3" t="str">
-        <v>media-1330.jpg</v>
+        <v>https://fouette.com.ar/</v>
+      </c>
+      <c r="L3" t="str">
+        <v>6.jpg</v>
+      </c>
+      <c r="M3">
+        <v>2</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Palestra</v>
+        <v>FOUETTE</v>
       </c>
       <c r="B4" t="str">
-        <v>palestra-santiago-de-los-caballero</v>
+        <v>Buenos Aires</v>
       </c>
       <c r="C4" t="str">
-        <v>republica-dominicana</v>
+        <v>fouette-buenos-aires</v>
       </c>
       <c r="D4" t="str">
-        <v>Ave. Juan Pablo Duarte, Centro Plaza Internacional 2do Nivel, Mod. 102</v>
+        <v>argentina</v>
       </c>
       <c r="E4" t="str">
-        <v/>
+        <v>Viamonte, 1177 (1053) – Cap. Fed.</v>
       </c>
       <c r="F4" t="str">
-        <v>(809) 841-2010</v>
+        <v>https://www.google.com/maps/place/FOUETTE/@-34.6003997,-58.3835588,3a,75y,320.29h,91.59t/data=!3m6!1e1!3m4!1sjz1sTnmoBFKtHjZL204GUg!2e0!7i16384!8i8192!4m16!1m9!3m8!1s0x95bccac7d473326f:0xa54ea16bec298df1!2sViamonte+1177,+C1053ABW+Cdad.+Aut%C3%B3noma+de+Buenos+Aires,+Argentina!3b1!8m2!3d-34.6003047!4d-58.3835845!10e5!16s%2Fg%2F11c5c49hth!3m5!1s0x95bccac7d473326f:0x72f4b58c49784070!8m2!3d-34.6003114!4d-58.3835836!16s%2Fg%2F11b6jh29ll?coh=205409&amp;entry=ttu&amp;g_ep=EgoyMDI0MTAwMi4xIKXMDSoASAFQAw%3D%3D</v>
       </c>
       <c r="G4" t="str">
-        <v>jocelynrodriguez@yahoo.com</v>
+        <v>+54 911 5723 7944</v>
       </c>
       <c r="H4" t="str">
-        <v/>
+        <v>ventas@32fouette.com.ar</v>
       </c>
       <c r="I4" t="str">
-        <v/>
-      </c>
-      <c r="J4" t="str">
-        <v/>
+        <v>https://www.instagram.com/fouette_32/</v>
       </c>
       <c r="K4" t="str">
-        <v>media-1326.jpg</v>
+        <v>https://fouette.com.ar/</v>
+      </c>
+      <c r="L4" t="str">
+        <v>5.jpg</v>
+      </c>
+      <c r="M4">
+        <v>3</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Sur la Pointe</v>
+        <v>Sara Nieto Dance</v>
       </c>
       <c r="B5" t="str">
-        <v>sur-la-pointe-ciudad-del-este</v>
+        <v>Viña Del Mar</v>
       </c>
       <c r="C5" t="str">
-        <v>paraguay</v>
+        <v>sara-nieto-dance-vina-del-mar</v>
       </c>
       <c r="D5" t="str">
-        <v>F9GJ+22J, Eugenio A. Garay, Cd. del Este 100151</v>
+        <v>chile</v>
       </c>
       <c r="E5" t="str">
-        <v>https://www.google.com/maps/place/Sur+La+Pointe.+Art%C3%ADculos+p%2F+danza/@-25.5249171,-54.6199787,17z/data=!3m1!4b1!4m6!3m5!1s0x94f68fee3c43aa39:0x45c48ee003c2b323!8m2!3d-25.5249171!4d-54.6199787!16s%2Fg%2F11bzq3j0nv?hl=en-PY&amp;entry=ttu&amp;g_ep=EgoyMDI0MTAxNC4wIKXMDSoASAFQAw%3D%3D</v>
+        <v>3 Ote. 1341, Local B, 2530904 Viña del Mar, Valparaíso, Chile</v>
       </c>
       <c r="F5" t="str">
-        <v>+595 982 706993</v>
+        <v>https://www.google.cl/maps/place/Tienda+Sara+Nieto+Vi%C3%B1a+del+Mar/@-33.0094641,-71.5495611,17z/data=!3m1!4b1!4m5!3m4!1s0x9689ddc259a325a1:0x82ad2c811c54c1cb!8m2!3d-33.0094687!4d-71.5450818</v>
       </c>
       <c r="G5" t="str">
-        <v>surlapointe.py@gmail.com</v>
-      </c>
-      <c r="H5" t="str">
-        <v/>
+        <v>+56322157850</v>
       </c>
       <c r="I5" t="str">
-        <v/>
+        <v>https://www.instagram.com/sodancachile/</v>
       </c>
       <c r="J5" t="str">
-        <v>https://www.surlapointe.com.py/</v>
+        <v>https://www.facebook.com/TiendasSaraNieto</v>
       </c>
       <c r="K5" t="str">
-        <v>media-1351.jpg</v>
+        <v>https://tiendasaranieto.cl/</v>
+      </c>
+      <c r="L5" t="str">
+        <v>15.jpg</v>
+      </c>
+      <c r="M5">
+        <v>1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Sur la Pointe</v>
+        <v>Sara Nieto Dance</v>
       </c>
       <c r="B6" t="str">
-        <v>sur-la-pointe-fdo-de-la-mora</v>
+        <v>Santiago Centro</v>
       </c>
       <c r="C6" t="str">
-        <v>paraguay</v>
+        <v>sara-nieto-dance-santiago-centro</v>
       </c>
       <c r="D6" t="str">
-        <v>Usher Ríos 171, Fernando de la Mora 110308</v>
+        <v>chile</v>
       </c>
       <c r="E6" t="str">
-        <v>https://www.google.com/maps/place/Sur+La+Pointe+Fdo+de+la+Mora/@-25.3245976,-57.5547844,17z/data=!3m1!4b1!4m6!3m5!1s0x945daed47c1554c5:0x63b40334337d05d2!8m2!3d-25.3245976!4d-57.5547844!16s%2Fg%2F11dxb17fzf?hl=en-PY&amp;entry=ttu&amp;g_ep=EgoyMDI0MTAxNC4wIKXMDSoASAFQAw%3D%3D</v>
+        <v>San Antonio 252, 8320202 Santiago, Región Metropolitana, Chile</v>
       </c>
       <c r="F6" t="str">
-        <v>+595 982 706938</v>
+        <v>https://www.google.cl/maps/place/Sara+Nieto/@-33.43767,-70.6419708,15z/data=!4m6!3m5!1s0x9662c5a3cd729cfd:0x8f84cbf445359193!8m2!3d-33.4399667!4d-70.6482!16s%2Fg%2F1vntl2cq?entry=ttu&amp;g_ep=EgoyMDI0MTAxNC4wIKXMDSoASAFQAw%3D%3D</v>
       </c>
       <c r="G6" t="str">
-        <v>surlapointe.py@gmail.com</v>
-      </c>
-      <c r="H6" t="str">
-        <v/>
+        <v>+56226399472</v>
       </c>
       <c r="I6" t="str">
-        <v/>
+        <v>https://www.instagram.com/sodancachile/</v>
       </c>
       <c r="J6" t="str">
-        <v>https://www.surlapointe.com.py/</v>
+        <v>https://www.facebook.com/TiendasSaraNieto</v>
       </c>
       <c r="K6" t="str">
-        <v>media-1350.jpg</v>
+        <v>https://tiendasaranieto.cl/</v>
+      </c>
+      <c r="L6" t="str">
+        <v>14.jpg</v>
+      </c>
+      <c r="M6">
+        <v>2</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Sur la Pointe - Centro</v>
+        <v>Sara Nieto Dance</v>
       </c>
       <c r="B7" t="str">
-        <v>sur-la-pointe-asuncion-centro</v>
+        <v>Academia</v>
       </c>
       <c r="C7" t="str">
-        <v>paraguay</v>
+        <v>sara-nieto-dance-academia</v>
       </c>
       <c r="D7" t="str">
-        <v>Colón 736, Asunción 001012</v>
+        <v>chile</v>
       </c>
       <c r="E7" t="str">
-        <v>https://www.google.com/maps/place/Sur+La+Pointe+Centro/@-25.2813576,-57.6437188,17z/data=!3m1!4b1!4m6!3m5!1s0x945da7ce4a9df027:0xa6c1c73761d24cde!8m2!3d-25.2813576!4d-57.6437188!16s%2Fg%2F11c2kn7kq9?hl=en-PY&amp;entry=ttu&amp;g_ep=EgoyMDI0MTAxNC4wIKXMDSoASAFQAw%3D%3D</v>
+        <v>Cerro Colorado 5030, L.3, Las Condes</v>
       </c>
       <c r="F7" t="str">
-        <v>+595 982 706222</v>
-      </c>
-      <c r="G7" t="str">
-        <v>surlapointe.py@gmail.com</v>
-      </c>
-      <c r="H7" t="str">
-        <v/>
+        <v>https://www.google.cl/maps/place/Cerro+Colorado+5030,+Las+Condes,+Regi%C3%B3n+Metropolitana,+Chile/@-33.4034777,-70.5812017,18z/data=!4m6!3m5!1s0x9662cf25dffb4159:0xa57007edd55798be!8m2!3d-33.4036685!4d-70.5799429!16s%2Fg%2F11dztskv15?entry=ttu&amp;g_ep=EgoyMDI0MTAxNC4wIKXMDSoASAFQAw%3D%3D</v>
       </c>
       <c r="I7" t="str">
-        <v/>
+        <v>https://www.instagram.com/sodancachile/</v>
       </c>
       <c r="J7" t="str">
-        <v>https://www.surlapointe.com.py/</v>
+        <v>https://www.facebook.com/TiendasSaraNieto</v>
       </c>
       <c r="K7" t="str">
-        <v>media-1349.jpg</v>
+        <v>https://tiendasaranieto.cl/</v>
+      </c>
+      <c r="L7" t="str">
+        <v>13.jpg</v>
+      </c>
+      <c r="M7">
+        <v>3</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Sur la Pointe - Lillo</v>
+        <v>Sara Nieto Dance</v>
       </c>
       <c r="B8" t="str">
-        <v>sur-la-pointe-asuncion-lillo</v>
+        <v>Apumanque</v>
       </c>
       <c r="C8" t="str">
-        <v>paraguay</v>
+        <v>sara-nieto-dance-apumanque</v>
       </c>
       <c r="D8" t="str">
-        <v>1459, Eusebio Lillo Robles, Asunción</v>
+        <v>chile</v>
       </c>
       <c r="E8" t="str">
-        <v>https://www.google.com/maps/place/Sur+La+Pointe/@-25.2888713,-57.5752319,17z/data=!3m1!4b1!4m6!3m5!1s0x945da8a1e604b5ef:0xc2c7e2c342094f7b!8m2!3d-25.2888713!4d-57.5752319!16s%2Fg%2F11c1ty51fg?hl=en-PY&amp;entry=ttu&amp;g_ep=EgoyMDI0MTAxNC4wIKXMDSoASAFQAw%3D%3D</v>
+        <v>Local 500, Apumanque, Av. Manquehue Sur 31, 7580001 Las Condes, Región Metropolitana, Chile</v>
       </c>
       <c r="F8" t="str">
-        <v>+595 982 706480</v>
+        <v>https://www.google.cl/maps/place/Store+Sara+Nieto+Apumanque/@-33.413934,-70.552809,12.75z/data=!4m6!3m5!1s0x9662ceddc3a12b4b:0x2985247702113939!8m2!3d-33.409534!4d-70.567352!16s%2Fg%2F1tt0sb3r?entry=ttu&amp;g_ep=EgoyMDI0MTAxNC4wIKXMDSoASAFQAw%3D%3D</v>
       </c>
       <c r="G8" t="str">
-        <v>surlapointe.py@gmail.com</v>
-      </c>
-      <c r="H8" t="str">
-        <v/>
+        <v>+56 9 7489 3344</v>
       </c>
       <c r="I8" t="str">
-        <v/>
+        <v>https://www.instagram.com/sodancachile/</v>
       </c>
       <c r="J8" t="str">
-        <v>https://www.surlapointe.com.py/</v>
+        <v>https://www.facebook.com/TiendasSaraNieto</v>
       </c>
       <c r="K8" t="str">
-        <v>media-1348.jpg</v>
+        <v>https://tiendasaranieto.cl/</v>
+      </c>
+      <c r="L8" t="str">
+        <v>12.jpg</v>
+      </c>
+      <c r="M8">
+        <v>4</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Cositas de Baile</v>
+        <v>In Dance - Sta Barbara</v>
       </c>
       <c r="B9" t="str">
-        <v>cositas-de-baile-panama-city</v>
+        <v>Bogotá</v>
       </c>
       <c r="C9" t="str">
-        <v>panama</v>
+        <v>in-dance-sta-barbara-bogota</v>
       </c>
       <c r="D9" t="str">
-        <v>C. 75 Este, Panamá, Provincia de Panamá, Panama</v>
+        <v>colombia</v>
       </c>
       <c r="E9" t="str">
-        <v>https://www.google.com/maps/@8.9911144,-79.5035001,3a,75y,158.62h,90t/data=!3m7!1e1!3m5!1shphk5izNzZ-DKrMbsTRvow!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D0%26panoid%3Dhphk5izNzZ-DKrMbsTRvow%26yaw%3D158.6207!7i16384!8i8192?coh=205410&amp;entry=ttu&amp;g_ep=EgoyMDI0MTAxNC4wIKXMDSoASAFQAw%3D%3D</v>
+        <v>Zona D diagonal a Dollarcity, Cra. 7 #115 - 60 Local D347 3 piso, Usaquén, Bogotá, Cundinamarca, Colombia</v>
       </c>
       <c r="F9" t="str">
-        <v>+507 6245-2000</v>
+        <v>https://www.google.com/maps/place/Indance+Sta+Barbara/@4.6922652,-74.0321922,17z/data=!3m1!4b1!4m6!3m5!1s0x8e3f9bacebe9e3cb:0xb1e1d4c7c1c3c9ae!8m2!3d4.6922652!4d-74.0321922!16s%2Fg%2F11ks20gqrx?entry=ttu&amp;g_ep=EgoyMDI0MTAxMy4wIKXMDSoASAFQAw%3D%3D</v>
       </c>
       <c r="G9" t="str">
-        <v>cositasdebailepanama@gmail.com</v>
+        <v>+57 310 2012221</v>
       </c>
       <c r="H9" t="str">
-        <v/>
+        <v>moveindance@gmail.com</v>
       </c>
       <c r="I9" t="str">
-        <v/>
-      </c>
-      <c r="J9" t="str">
-        <v>https://www.cositasdebaile.com/</v>
-      </c>
-      <c r="K9" t="str">
-        <v>media-1353.jpg</v>
+        <v>https://www.instagram.com/indanceco/</v>
+      </c>
+      <c r="L9" t="str">
+        <v>9.jpg</v>
+      </c>
+      <c r="M9">
+        <v>1</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Dance Shoes - San Pedro Sula</v>
+        <v>In Dance - Centro</v>
       </c>
       <c r="B10" t="str">
-        <v>dance-shoes-san-pedro-sula</v>
+        <v>Bogotá</v>
       </c>
       <c r="C10" t="str">
-        <v/>
+        <v>in-dance-centro-bogota</v>
       </c>
       <c r="D10" t="str">
-        <v>Colonia Satelite Calle Principal Casa 806 Bloque 10</v>
+        <v>colombia</v>
       </c>
       <c r="E10" t="str">
-        <v/>
+        <v>Centro Comercial Galerias, Local 1081, Cra 27 #Calle 54 Entrada 7, Bogotá, Colombia</v>
       </c>
       <c r="F10" t="str">
-        <v>(504) 9729-0226</v>
+        <v>https://www.google.com/maps/place/InDance+-+Tu+Tienda+de+Danza+-+galerias/@4.6433196,-74.075819,17z/data=!3m1!4b1!4m6!3m5!1s0x8e3f9a34f3b5110f:0xf6a4708ffeab58ab!8m2!3d4.6433196!4d-74.075819!16s%2Fg%2F1ptzq7v60?entry=ttu&amp;g_ep=EgoyMDI0MTAxMy4wIKXMDSoASAFQAw%3D%3D</v>
       </c>
       <c r="G10" t="str">
-        <v>dance_shoes504@hotmail.com</v>
+        <v>+57 310 2012221</v>
       </c>
       <c r="H10" t="str">
-        <v/>
+        <v>mkt@indance.com.co</v>
       </c>
       <c r="I10" t="str">
-        <v/>
-      </c>
-      <c r="J10" t="str">
-        <v/>
-      </c>
-      <c r="K10" t="str">
-        <v/>
+        <v>https://www.instagram.com/indanceco/</v>
+      </c>
+      <c r="L10" t="str">
+        <v>8.jpg</v>
+      </c>
+      <c r="M10">
+        <v>2</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Joy Dance</v>
+        <v>DanceCo Boutique</v>
       </c>
       <c r="B11" t="str">
-        <v>joy-dance-guatemala-city</v>
+        <v>San José</v>
       </c>
       <c r="C11" t="str">
-        <v>guatemala</v>
+        <v>danceco-boutique-san-jose</v>
       </c>
       <c r="D11" t="str">
-        <v>18 calle 10-50 zona 10 Centro Comercial La Villa 01010</v>
+        <v>costa-rica</v>
       </c>
       <c r="E11" t="str">
-        <v/>
-      </c>
-      <c r="F11" t="str">
-        <v>+502 2367 6831</v>
+        <v>Sabana Sur 125 este de la Pops+506 2290 2913 / +506 8815 3761[email protected]Instagram</v>
       </c>
       <c r="G11" t="str">
-        <v>joydanceandactivewear@gmail.com</v>
+        <v>+506 2290 2913 / +506 8815 3761</v>
       </c>
       <c r="H11" t="str">
-        <v/>
+        <v>ventas@danceco.co.cr</v>
       </c>
       <c r="I11" t="str">
-        <v/>
-      </c>
-      <c r="J11" t="str">
-        <v>https://joydanceandactivewear.com/</v>
-      </c>
-      <c r="K11" t="str">
-        <v>media-1304.png</v>
+        <v>https://www.instagram.com/danceco_boutique/</v>
+      </c>
+      <c r="L11" t="str">
+        <v>4.jpg</v>
+      </c>
+      <c r="M11">
+        <v>1</v>
       </c>
     </row>
     <row r="12">
@@ -944,564 +965,568 @@
         <v>Jeté</v>
       </c>
       <c r="B12" t="str">
+        <v>Quito</v>
+      </c>
+      <c r="C12" t="str">
         <v>jete-quito</v>
       </c>
-      <c r="C12" t="str">
+      <c r="D12" t="str">
         <v>ecuador</v>
       </c>
-      <c r="D12" t="str">
-        <v>Tamayo N24-535 Y Luis Cordero 170523</v>
-      </c>
       <c r="E12" t="str">
-        <v/>
-      </c>
-      <c r="F12" t="str">
+        <v>Tamayo N24-535 Y Luis Cordero 170523+593 99 537 0224[email protected]Facebook</v>
+      </c>
+      <c r="G12" t="str">
         <v>+593 99 537 0224</v>
       </c>
-      <c r="G12" t="str">
+      <c r="H12" t="str">
         <v>paty660303@hotmail.com</v>
       </c>
-      <c r="H12" t="str">
-        <v/>
-      </c>
-      <c r="I12" t="str">
-        <v/>
-      </c>
       <c r="J12" t="str">
-        <v/>
-      </c>
-      <c r="K12" t="str">
-        <v>media-1301.jpg</v>
+        <v>https://www.facebook.com/jete.sodanca.ec/</v>
+      </c>
+      <c r="L12" t="str">
+        <v>305934810_509394084524854_5312535576866439499_n.jpg</v>
+      </c>
+      <c r="M12">
+        <v>1</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>DanceCo Boutique</v>
+        <v>Joy Dance</v>
       </c>
       <c r="B13" t="str">
-        <v>danceco-boutique-san-jose</v>
+        <v>Guatemala City</v>
       </c>
       <c r="C13" t="str">
-        <v>costa-rica</v>
+        <v>joy-dance-guatemala-city</v>
       </c>
       <c r="D13" t="str">
-        <v>Sabana Sur 125 este de la Pops</v>
+        <v>guatemala</v>
       </c>
       <c r="E13" t="str">
-        <v/>
-      </c>
-      <c r="F13" t="str">
-        <v>+506 2290 2913 / +506 8815 3761</v>
+        <v>18 calle 10-50 zona 10 Centro Comercial La Villa 01010+502 2367 6831[email protected]InstagramFacebook</v>
       </c>
       <c r="G13" t="str">
-        <v>ventas@danceco.co.cr</v>
+        <v>+502 2367 6831</v>
       </c>
       <c r="H13" t="str">
-        <v/>
+        <v>joydanceandactivewear@gmail.com</v>
       </c>
       <c r="I13" t="str">
-        <v/>
+        <v>https://www.instagram.com/joydanceandactivewear/</v>
       </c>
       <c r="J13" t="str">
-        <v/>
+        <v>https://www.facebook.com/joydanceandactivewear/</v>
       </c>
       <c r="K13" t="str">
-        <v>media-1344.jpg</v>
+        <v>https://joydanceandactivewear.com/</v>
+      </c>
+      <c r="L13" t="str">
+        <v>326561771_503577385230999_6516429715477023224_n.png</v>
+      </c>
+      <c r="M13">
+        <v>1</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>In Dance - Sta Barbara</v>
+        <v>Pirouette</v>
       </c>
       <c r="B14" t="str">
-        <v>in-dance-sta-barbara</v>
+        <v>Guadalajara</v>
       </c>
       <c r="C14" t="str">
-        <v>colombia</v>
+        <v>pirouette-guadalajara</v>
       </c>
       <c r="D14" t="str">
-        <v>Zona D diagonal a Dollarcity, Cra. 7 #115 - 60 Local D347 3 piso, Usaquén, Bogotá, Cundinamarca, Colombia</v>
+        <v>mexico</v>
       </c>
       <c r="E14" t="str">
-        <v>https://www.google.com/maps/place/Indance+Sta+Barbara/@4.6922652,-74.0321922,17z/data=!3m1!4b1!4m6!3m5!1s0x8e3f9bacebe9e3cb:0xb1e1d4c7c1c3c9ae!8m2!3d4.6922652!4d-74.0321922!16s%2Fg%2F11ks20gqrx?entry=ttu&amp;g_ep=EgoyMDI0MTAxMy4wIKXMDSoASAFQAw%3D%3D</v>
-      </c>
-      <c r="F14" t="str">
-        <v>+57 310 2012221</v>
+        <v>Plaza Universidad, Local G-4 (Pablo Neruda #4341, esquina con Av. Patria)+52 33 3610 0291[email protected]Instagram</v>
       </c>
       <c r="G14" t="str">
-        <v>moveindance@gmail.com</v>
+        <v>+52 33 3610 0291</v>
       </c>
       <c r="H14" t="str">
-        <v/>
+        <v>mariana_fv01@hotmail.com</v>
       </c>
       <c r="I14" t="str">
-        <v/>
-      </c>
-      <c r="J14" t="str">
-        <v/>
-      </c>
-      <c r="K14" t="str">
-        <v>media-1343.jpg</v>
+        <v>https://www.instagram.com/pirouettetienda/</v>
+      </c>
+      <c r="L14" t="str">
+        <v>Punta-Carretas-2.jpg</v>
+      </c>
+      <c r="M14">
+        <v>1</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>In Dance - Centro</v>
+        <v>Andanzza</v>
       </c>
       <c r="B15" t="str">
-        <v>in-dance-bogota</v>
+        <v>Edo México</v>
       </c>
       <c r="C15" t="str">
-        <v>colombia</v>
+        <v>andanzza-edo-mexico</v>
       </c>
       <c r="D15" t="str">
-        <v>Centro Comercial Galerias, Local 1081, Cra 27 #Calle 54 Entrada 7, Bogotá, Colombia</v>
+        <v>mexico</v>
       </c>
       <c r="E15" t="str">
-        <v>https://www.google.com/maps/place/InDance+-+Tu+Tienda+de+Danza+-+galerias/@4.6433196,-74.075819,17z/data=!3m1!4b1!4m6!3m5!1s0x8e3f9a34f3b5110f:0xf6a4708ffeab58ab!8m2!3d4.6433196!4d-74.075819!16s%2Fg%2F1ptzq7v60?entry=ttu&amp;g_ep=EgoyMDI0MTAxMy4wIKXMDSoASAFQAw%3D%3D</v>
+        <v>Blvd. Interlomas #5 Col. La Herradura Huixquilucan, 52786, Edo México</v>
       </c>
       <c r="F15" t="str">
-        <v>+57 310 2012221</v>
-      </c>
-      <c r="G15" t="str">
-        <v>mkt@indance.com.co</v>
+        <v>https://www.google.com/maps/place/Andanzza+Interlomas/@19.4019735,-99.2698902,17z/data=!3m1!4b1!4m6!3m5!1s0x85d20742eff15e35:0xd145553d5df10d8d!8m2!3d19.4019735!4d-99.2698902!16s%2Fg%2F1tjl67ts?entry=ttu&amp;g_ep=EgoyMDI0MTAxMy4wIKXMDSoASAFQAw%3D%3D</v>
       </c>
       <c r="H15" t="str">
-        <v/>
+        <v>ventas@andanzza.com.mx</v>
       </c>
       <c r="I15" t="str">
-        <v/>
+        <v>https://www.instagram.com/andanzzamx/</v>
       </c>
       <c r="J15" t="str">
-        <v/>
+        <v>https://www.facebook.com/AndanzzaMX/</v>
       </c>
       <c r="K15" t="str">
-        <v>media-1342.jpg</v>
+        <v>https://andanzza.com.mx/</v>
+      </c>
+      <c r="L15" t="str">
+        <v>4-1.jpg</v>
+      </c>
+      <c r="M15">
+        <v>2</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Sara Nieto Dance</v>
+        <v>Andanzza</v>
       </c>
       <c r="B16" t="str">
-        <v>sara-nieto-dance-vina-del-mar</v>
+        <v>Ciudad de México</v>
       </c>
       <c r="C16" t="str">
-        <v>chile</v>
+        <v>andanzza-ciudad-de-mexico</v>
       </c>
       <c r="D16" t="str">
-        <v>3 Ote. 1341, Local B, 2530904 Viña del Mar, Valparaíso, Chile</v>
+        <v>mexico</v>
       </c>
       <c r="E16" t="str">
-        <v>https://www.google.cl/maps/place/Tienda+Sara+Nieto+Vi%C3%B1a+del+Mar/@-33.0094641,-71.5495611,17z/data=!3m1!4b1!4m5!3m4!1s0x9689ddc259a325a1:0x82ad2c811c54c1cb!8m2!3d-33.0094687!4d-71.5450818</v>
+        <v>Prado Sur #146 piso 2 Col. Lomas de Chapultepec Miguel Hidalgo, 11000, CDMX</v>
       </c>
       <c r="F16" t="str">
-        <v>+56322157850</v>
-      </c>
-      <c r="G16" t="str">
-        <v/>
+        <v>https://www.google.com/maps/place/Andanzza+Lomas+(Prado+Sur)/@19.425861,-99.2048622,17z/data=!3m1!4b1!4m6!3m5!1s0x85d2021943e859a3:0xcd1f076d98ea1daf!8m2!3d19.425861!4d-99.2048622!16s%2Fg%2F1ptx3qgwl?entry=ttu&amp;g_ep=EgoyMDI0MTAxMy4wIKXMDSoASAFQAw%3D%3D</v>
       </c>
       <c r="H16" t="str">
-        <v/>
+        <v>ventas@andanzza.com.mx</v>
       </c>
       <c r="I16" t="str">
-        <v/>
+        <v>https://www.instagram.com/andanzzamx/</v>
       </c>
       <c r="J16" t="str">
-        <v>https://tiendasaranieto.cl/</v>
+        <v>https://www.facebook.com/AndanzzaMX/</v>
       </c>
       <c r="K16" t="str">
-        <v>media-1341.jpg</v>
+        <v>https://andanzza.com.mx/</v>
+      </c>
+      <c r="L16" t="str">
+        <v>3.jpg</v>
+      </c>
+      <c r="M16">
+        <v>3</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Sara Nieto Dance</v>
+        <v>Petipá</v>
       </c>
       <c r="B17" t="str">
-        <v>sara-nieto-dance-santiago-centro</v>
+        <v>Ciudad de México</v>
       </c>
       <c r="C17" t="str">
-        <v>chile</v>
+        <v>petipa-ciudad-de-mexico</v>
       </c>
       <c r="D17" t="str">
-        <v>San Antonio 252, 8320202 Santiago, Región Metropolitana, Chile</v>
+        <v>mexico</v>
       </c>
       <c r="E17" t="str">
-        <v>https://www.google.cl/maps/place/Sara+Nieto/@-33.43767,-70.6419708,15z/data=!4m6!3m5!1s0x9662c5a3cd729cfd:0x8f84cbf445359193!8m2!3d-33.4399667!4d-70.6482!16s%2Fg%2F1vntl2cq?entry=ttu&amp;g_ep=EgoyMDI0MTAxNC4wIKXMDSoASAFQAw%3D%3D</v>
+        <v>Miguel Ángel Miguel Angel de Quevedo #140 local 6</v>
       </c>
       <c r="F17" t="str">
-        <v>+56226399472</v>
+        <v>https://www.google.com/maps/place/Petipa+MAQ/@19.347401,-99.1817931,3a,75y,353.61h,90.33t/data=!3m8!1e1!3m5!1spV-sei-naXWZKbgj49aw6w!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-0.3341314013255925%26panoid%3DpV-sei-naXWZKbgj49aw6w%26yaw%3D353.60959930407415!7i16384!8i8192!5s0x85d1fffa626a4707:0xaa1bc8f0213af215!4m6!3m5!1s0x85d1fffa63023daf:0xc20267c62dfc442d!8m2!3d19.3475804!4d-99.1817521!16s%2Fg%2F1tf3zqcc?coh=205410&amp;entry=ttu&amp;g_ep=EgoyMDI0MTAwMi4xIKXMDSoASAFQAw%3D%3D</v>
       </c>
       <c r="G17" t="str">
-        <v/>
+        <v>+52 55 5662-0210</v>
       </c>
       <c r="H17" t="str">
-        <v/>
+        <v>petipa_nancyalvarado@hotmail.com</v>
       </c>
       <c r="I17" t="str">
-        <v/>
+        <v>https://www.instagram.com/petipamexico/</v>
       </c>
       <c r="J17" t="str">
-        <v>https://tiendasaranieto.cl/</v>
+        <v>https://www.facebook.com/Petipamx</v>
       </c>
       <c r="K17" t="str">
-        <v>media-1340.jpg</v>
+        <v>https://tiendapetipa.com/</v>
+      </c>
+      <c r="L17" t="str">
+        <v>456263623_1044437404349624_7515373991471178028_n.jpg</v>
+      </c>
+      <c r="M17">
+        <v>4</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Sara Nieto Dance</v>
+        <v>Cositas de Baile</v>
       </c>
       <c r="B18" t="str">
-        <v>sara-nieto-dance-academia</v>
+        <v>Panama City</v>
       </c>
       <c r="C18" t="str">
-        <v>chile</v>
+        <v>cositas-de-baile-panama-city</v>
       </c>
       <c r="D18" t="str">
-        <v>Cerro Colorado 5030, L.3, Las Condes</v>
+        <v>panama</v>
       </c>
       <c r="E18" t="str">
-        <v>https://www.google.cl/maps/place/Cerro+Colorado+5030,+Las+Condes,+Regi%C3%B3n+Metropolitana,+Chile/@-33.4034777,-70.5812017,18z/data=!4m6!3m5!1s0x9662cf25dffb4159:0xa57007edd55798be!8m2!3d-33.4036685!4d-70.5799429!16s%2Fg%2F11dztskv15?entry=ttu&amp;g_ep=EgoyMDI0MTAxNC4wIKXMDSoASAFQAw%3D%3D</v>
+        <v>C. 75 Este, Panamá, Provincia de Panamá, Panama</v>
       </c>
       <c r="F18" t="str">
-        <v>223629792</v>
+        <v>https://www.google.com/maps/@8.9911144,-79.5035001,3a,75y,158.62h,90t/data=!3m7!1e1!3m5!1shphk5izNzZ-DKrMbsTRvow!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D0%26panoid%3Dhphk5izNzZ-DKrMbsTRvow%26yaw%3D158.6207!7i16384!8i8192?coh=205410&amp;entry=ttu&amp;g_ep=EgoyMDI0MTAxNC4wIKXMDSoASAFQAw%3D%3D</v>
       </c>
       <c r="G18" t="str">
-        <v/>
+        <v>+507 6245-2000</v>
       </c>
       <c r="H18" t="str">
-        <v/>
+        <v>cositasdebailepanama@gmail.com</v>
       </c>
       <c r="I18" t="str">
-        <v/>
+        <v>https://www.instagram.com/cositasdebaile/</v>
       </c>
       <c r="J18" t="str">
-        <v>https://tiendasaranieto.cl/</v>
+        <v>https://www.facebook.com/Cositasdebaile/</v>
       </c>
       <c r="K18" t="str">
-        <v>media-1339.jpg</v>
+        <v>https://www.cositasdebaile.com/</v>
+      </c>
+      <c r="L18" t="str">
+        <v>Punta-Carretas-1-1.jpg</v>
+      </c>
+      <c r="M18">
+        <v>1</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Sara Nieto Dance</v>
+        <v>Sur la Pointe</v>
       </c>
       <c r="B19" t="str">
-        <v>sara-nieto-dance-apumanque</v>
+        <v>Ciudad del Este</v>
       </c>
       <c r="C19" t="str">
-        <v>chile</v>
+        <v>sur-la-pointe-ciudad-del-este</v>
       </c>
       <c r="D19" t="str">
-        <v>Local 500, Apumanque, Av. Manquehue Sur 31, 7580001 Las Condes, Región Metropolitana, Chile</v>
+        <v>paraguay</v>
       </c>
       <c r="E19" t="str">
-        <v>https://www.google.cl/maps/place/Store+Sara+Nieto+Apumanque/@-33.413934,-70.552809,12.75z/data=!4m6!3m5!1s0x9662ceddc3a12b4b:0x2985247702113939!8m2!3d-33.409534!4d-70.567352!16s%2Fg%2F1tt0sb3r?entry=ttu&amp;g_ep=EgoyMDI0MTAxNC4wIKXMDSoASAFQAw%3D%3D</v>
+        <v>F9GJ+22J, Eugenio A. Garay, Cd. del Este 100151</v>
       </c>
       <c r="F19" t="str">
-        <v>+56 9 7489 3344</v>
+        <v>https://www.google.com/maps/place/Sur+La+Pointe.+Art%C3%ADculos+p%2F+danza/@-25.5249171,-54.6199787,17z/data=!3m1!4b1!4m6!3m5!1s0x94f68fee3c43aa39:0x45c48ee003c2b323!8m2!3d-25.5249171!4d-54.6199787!16s%2Fg%2F11bzq3j0nv?hl=en-PY&amp;entry=ttu&amp;g_ep=EgoyMDI0MTAxNC4wIKXMDSoASAFQAw%3D%3D</v>
       </c>
       <c r="G19" t="str">
-        <v/>
+        <v>+595 982 706993</v>
       </c>
       <c r="H19" t="str">
-        <v/>
+        <v>surlapointe.py@gmail.com</v>
       </c>
       <c r="I19" t="str">
-        <v/>
+        <v>https://www.instagram.com/surlapointeballet/</v>
       </c>
       <c r="J19" t="str">
-        <v>https://tiendasaranieto.cl/</v>
+        <v>https://www.facebook.com/SurlaPointePy</v>
       </c>
       <c r="K19" t="str">
-        <v>media-1338.jpg</v>
+        <v>https://www.surlapointe.com.py/</v>
+      </c>
+      <c r="L19" t="str">
+        <v>21.jpg</v>
+      </c>
+      <c r="M19">
+        <v>1</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Pirouette</v>
+        <v>Sur la Pointe</v>
       </c>
       <c r="B20" t="str">
-        <v>pirouette-guadalajara</v>
+        <v>Fdo de la Mora</v>
       </c>
       <c r="C20" t="str">
-        <v>mexico</v>
+        <v>sur-la-pointe-fdo-de-la-mora</v>
       </c>
       <c r="D20" t="str">
-        <v>Plaza Universidad, Local G-4 (Pablo Neruda #4341, esquina con Av. Patria)</v>
+        <v>paraguay</v>
       </c>
       <c r="E20" t="str">
-        <v/>
+        <v>Usher Ríos 171, Fernando de la Mora 110308</v>
       </c>
       <c r="F20" t="str">
-        <v>+52 33 3610 0291</v>
+        <v>https://www.google.com/maps/place/Sur+La+Pointe+Fdo+de+la+Mora/@-25.3245976,-57.5547844,17z/data=!3m1!4b1!4m6!3m5!1s0x945daed47c1554c5:0x63b40334337d05d2!8m2!3d-25.3245976!4d-57.5547844!16s%2Fg%2F11dxb17fzf?hl=en-PY&amp;entry=ttu&amp;g_ep=EgoyMDI0MTAxNC4wIKXMDSoASAFQAw%3D%3D</v>
       </c>
       <c r="G20" t="str">
-        <v>mariana_fv01@hotmail.com</v>
+        <v>+595 982 706938</v>
       </c>
       <c r="H20" t="str">
-        <v/>
+        <v>surlapointe.py@gmail.com</v>
       </c>
       <c r="I20" t="str">
-        <v/>
+        <v>https://www.instagram.com/surlapointeballet/</v>
       </c>
       <c r="J20" t="str">
-        <v/>
+        <v>https://www.facebook.com/SurlaPointePy</v>
       </c>
       <c r="K20" t="str">
-        <v>media-1347.jpg</v>
+        <v>https://www.surlapointe.com.py/</v>
+      </c>
+      <c r="L20" t="str">
+        <v>20.jpg</v>
+      </c>
+      <c r="M20">
+        <v>2</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Andanzza</v>
+        <v>Sur la Pointe - Centro</v>
       </c>
       <c r="B21" t="str">
-        <v>andanzza-dance-shop-interlomas-edo-mexico</v>
+        <v>Asunción</v>
       </c>
       <c r="C21" t="str">
-        <v>mexico</v>
+        <v>sur-la-pointe-centro-asuncion</v>
       </c>
       <c r="D21" t="str">
-        <v>Blvd. Interlomas #5 Col. La Herradura Huixquilucan, 52786, Edo México</v>
+        <v>paraguay</v>
       </c>
       <c r="E21" t="str">
-        <v>https://www.google.com/maps/place/Andanzza+Interlomas/@19.4019735,-99.2698902,17z/data=!3m1!4b1!4m6!3m5!1s0x85d20742eff15e35:0xd145553d5df10d8d!8m2!3d19.4019735!4d-99.2698902!16s%2Fg%2F1tjl67ts?entry=ttu&amp;g_ep=EgoyMDI0MTAxMy4wIKXMDSoASAFQAw%3D%3D</v>
+        <v>Colón 736, Asunción 001012</v>
       </c>
       <c r="F21" t="str">
-        <v>(55) 6155 8577</v>
+        <v>https://www.google.com/maps/place/Sur+La+Pointe+Centro/@-25.2813576,-57.6437188,17z/data=!3m1!4b1!4m6!3m5!1s0x945da7ce4a9df027:0xa6c1c73761d24cde!8m2!3d-25.2813576!4d-57.6437188!16s%2Fg%2F11c2kn7kq9?hl=en-PY&amp;entry=ttu&amp;g_ep=EgoyMDI0MTAxNC4wIKXMDSoASAFQAw%3D%3D</v>
       </c>
       <c r="G21" t="str">
-        <v>ventas@andanzza.com.mx</v>
+        <v>+595 982 706222</v>
       </c>
       <c r="H21" t="str">
-        <v/>
+        <v>surlapointe.py@gmail.com</v>
       </c>
       <c r="I21" t="str">
-        <v/>
+        <v>https://www.instagram.com/surlapointeballet/</v>
       </c>
       <c r="J21" t="str">
-        <v>https://andanzza.com.mx/</v>
+        <v>https://www.facebook.com/SurlaPointePy</v>
       </c>
       <c r="K21" t="str">
-        <v>media-1346.jpg</v>
+        <v>https://www.surlapointe.com.py/</v>
+      </c>
+      <c r="L21" t="str">
+        <v>19.jpg</v>
+      </c>
+      <c r="M21">
+        <v>3</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Andanzza</v>
+        <v>Sur la Pointe - Lillo</v>
       </c>
       <c r="B22" t="str">
-        <v>andanzza-dance-shop-ciudad-de-mexico</v>
+        <v>Asunción</v>
       </c>
       <c r="C22" t="str">
-        <v>mexico</v>
+        <v>sur-la-pointe-lillo-asuncion</v>
       </c>
       <c r="D22" t="str">
-        <v>Prado Sur #146 piso 2 Col. Lomas de Chapultepec Miguel Hidalgo, 11000, CDMX</v>
+        <v>paraguay</v>
       </c>
       <c r="E22" t="str">
-        <v>https://www.google.com/maps/place/Andanzza+Lomas+(Prado+Sur)/@19.425861,-99.2048622,17z/data=!3m1!4b1!4m6!3m5!1s0x85d2021943e859a3:0xcd1f076d98ea1daf!8m2!3d19.425861!4d-99.2048622!16s%2Fg%2F1ptx3qgwl?entry=ttu&amp;g_ep=EgoyMDI0MTAxMy4wIKXMDSoASAFQAw%3D%3D</v>
+        <v>1459, Eusebio Lillo Robles, Asunción</v>
       </c>
       <c r="F22" t="str">
-        <v>(55) 5580-5898</v>
+        <v>https://www.google.com/maps/place/Sur+La+Pointe/@-25.2888713,-57.5752319,17z/data=!3m1!4b1!4m6!3m5!1s0x945da8a1e604b5ef:0xc2c7e2c342094f7b!8m2!3d-25.2888713!4d-57.5752319!16s%2Fg%2F11c1ty51fg?hl=en-PY&amp;entry=ttu&amp;g_ep=EgoyMDI0MTAxNC4wIKXMDSoASAFQAw%3D%3D</v>
       </c>
       <c r="G22" t="str">
-        <v>ventas@andanzza.com.mx</v>
+        <v>+595 982 706480</v>
       </c>
       <c r="H22" t="str">
-        <v/>
+        <v>surlapointe.py@gmail.com</v>
       </c>
       <c r="I22" t="str">
-        <v/>
+        <v>https://www.instagram.com/surlapointeballet/</v>
       </c>
       <c r="J22" t="str">
-        <v>https://andanzza.com.mx/</v>
+        <v>https://www.facebook.com/SurlaPointePy</v>
       </c>
       <c r="K22" t="str">
-        <v>media-1345.jpg</v>
+        <v>https://www.surlapointe.com.py/</v>
+      </c>
+      <c r="L22" t="str">
+        <v>18.jpg</v>
+      </c>
+      <c r="M22">
+        <v>4</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Petipá</v>
+        <v>Palestra</v>
       </c>
       <c r="B23" t="str">
-        <v>petipa-miguel-angel-ciudad-de-mexico</v>
+        <v>Santiago de los Caballero</v>
       </c>
       <c r="C23" t="str">
-        <v>mexico</v>
+        <v>palestra-santiago-de-los-caballero</v>
       </c>
       <c r="D23" t="str">
-        <v>Miguel Ángel Miguel Angel de Quevedo #140 local 6</v>
+        <v>republica-dominicana</v>
       </c>
       <c r="E23" t="str">
-        <v>https://www.google.com/maps/place/Petipa+MAQ/@19.347401,-99.1817931,3a,75y,353.61h,90.33t/data=!3m8!1e1!3m5!1spV-sei-naXWZKbgj49aw6w!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-0.3341314013255925%26panoid%3DpV-sei-naXWZKbgj49aw6w%26yaw%3D353.60959930407415!7i16384!8i8192!5s0x85d1fffa626a4707:0xaa1bc8f0213af215!4m6!3m5!1s0x85d1fffa63023daf:0xc20267c62dfc442d!8m2!3d19.3475804!4d-99.1817521!16s%2Fg%2F1tf3zqcc?coh=205410&amp;entry=ttu&amp;g_ep=EgoyMDI0MTAwMi4xIKXMDSoASAFQAw%3D%3D</v>
-      </c>
-      <c r="F23" t="str">
-        <v>+52 55 5662-0210</v>
-      </c>
-      <c r="G23" t="str">
-        <v>petipa_nancyalvarado@hotmail.com</v>
+        <v>Ave. Juan Pablo Duarte, Centro Plaza Internacional 2do Nivel, Mod. 102(809) 841-2010[email protected]Instagram</v>
       </c>
       <c r="H23" t="str">
-        <v/>
+        <v>jocelynrodriguez@yahoo.com</v>
       </c>
       <c r="I23" t="str">
-        <v/>
-      </c>
-      <c r="J23" t="str">
-        <v>https://tiendapetipa.com/</v>
+        <v>https://www.instagram.com/sodancard/</v>
       </c>
       <c r="K23" t="str">
-        <v>media-1278.jpg</v>
+        <v>http://(809)%20841-2010</v>
+      </c>
+      <c r="L23" t="str">
+        <v>Design-sem-nome-2.jpg</v>
+      </c>
+      <c r="M23">
+        <v>1</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Volé</v>
+        <v>The Dance Shop</v>
       </c>
       <c r="B24" t="str">
-        <v>vole-valencia-carabobo</v>
+        <v>Montevideo C.</v>
       </c>
       <c r="C24" t="str">
-        <v>venezuela</v>
+        <v>the-dance-shop-montevideo-c</v>
       </c>
       <c r="D24" t="str">
-        <v>C.C Multicentro El Viñedo, Valencia</v>
+        <v>uruguay</v>
       </c>
       <c r="E24" t="str">
-        <v>https://www.google.com/maps/place/Multicentre+Vineyard/@10.2094622,-68.00859,16.25z/data=!4m6!3m5!1s0x8e805d9a4ddaf96b:0x6cd0bb2174ab91b7!8m2!3d10.2131461!4d-68.0093357!16s%2Fg%2F1hm4cgzwy?entry=ttu&amp;g_ep=EgoyMDI0MTAwMi4xIKXMDSoASAFQAw%3D%3D</v>
-      </c>
-      <c r="F24" t="str">
-        <v>+58 412-4330767</v>
+        <v>Carlos Sáez y Arocena, Galeria Roma Local 1+598 91 463 106[email protected]Instagram</v>
       </c>
       <c r="G24" t="str">
-        <v>volevenezuela@gmail.com</v>
+        <v>+598 91 463 106</v>
       </c>
       <c r="H24" t="str">
-        <v/>
+        <v>danceshop.uy@gmail.com</v>
       </c>
       <c r="I24" t="str">
-        <v/>
-      </c>
-      <c r="J24" t="str">
-        <v>https://treinta.shop/vol-a47b97</v>
+        <v>https://www.instagram.com/thedanceshopuy/</v>
       </c>
       <c r="K24" t="str">
-        <v>media-1352.jpg</v>
+        <v>https://thedanceshop.com.uy/</v>
+      </c>
+      <c r="L24" t="str">
+        <v>Punta-Carretas-1.jpg</v>
+      </c>
+      <c r="M24">
+        <v>1</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>FOUETTE</v>
+        <v>The Dance Shop</v>
       </c>
       <c r="B25" t="str">
-        <v>fouette-mendoza</v>
+        <v>Montevideo P.C</v>
       </c>
       <c r="C25" t="str">
-        <v>argentina</v>
+        <v>the-dance-shop-montevideo-pc</v>
       </c>
       <c r="D25" t="str">
-        <v>Lavalle 35/45 local 34 Galería Independencia - Mendoza Capital</v>
+        <v>uruguay</v>
       </c>
       <c r="E25" t="str">
-        <v>https://www.google.com/maps/place/Galer%C3%ADa+Independencia/@-32.8885556,-68.8380256,3a,75y,157.02h,91.78t/data=!3m7!1e1!3m5!1s8tSur1-aHdwxmAjLuXr1YA!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-1.7792920309981781%26panoid%3D8tSur1-aHdwxmAjLuXr1YA%26yaw%3D157.02122739013302!7i16384!8i8192!4m14!1m7!3m6!1s0x967e091906ac3fb5:0xd1f38edf52822e93!2sGaler%C3%ADa+Independencia!8m2!3d-32.8890198!4d-68.8381173!16s%2Fg%2F11bw4hy0dt!3m5!1s0x967e091906ac3fb5:0xd1f38edf52822e93!8m2!3d-32.8890198!4d-68.8381173!16s%2Fg%2F11bw4hy0dt?coh=205410&amp;entry=ttu&amp;g_ep=EgoyMDI0MTAwMi4xIKXMDSoASAFQAw%3D%3D</v>
-      </c>
-      <c r="F25" t="str">
-        <v>+54 911 5724-1569</v>
+        <v>21 de setiembre 2951, esq. Tomás Diago+598 91 463 106[email protected]Instagram</v>
       </c>
       <c r="G25" t="str">
-        <v>ventas@32fouette.com.ar</v>
+        <v>+598 91 463 106</v>
       </c>
       <c r="H25" t="str">
-        <v/>
+        <v>danceshop.uy@gmail.com</v>
       </c>
       <c r="I25" t="str">
-        <v/>
-      </c>
-      <c r="J25" t="str">
-        <v>https://fouette.com.ar/</v>
+        <v>https://www.instagram.com/thedanceshopuy/</v>
       </c>
       <c r="K25" t="str">
-        <v>media-1337.jpg</v>
+        <v>https://thedanceshop.com.uy/</v>
+      </c>
+      <c r="L25" t="str">
+        <v>Punta-Carretas.jpg</v>
+      </c>
+      <c r="M25">
+        <v>2</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>FOUETTE</v>
+        <v>Volé</v>
       </c>
       <c r="B26" t="str">
-        <v>fouette-cordoba</v>
+        <v>Valencia, Carabobo</v>
       </c>
       <c r="C26" t="str">
-        <v>argentina</v>
+        <v>vole-valencia-carabobo</v>
       </c>
       <c r="D26" t="str">
-        <v>Córdoba 3068, Mar del Plata</v>
+        <v>venezuela</v>
       </c>
       <c r="E26" t="str">
-        <v>https://www.google.com/maps/place/Fouette/@-38.0103675,-57.5557138,3a,75y,115.85h,95.65t/data=!3m7!1e1!3m5!1srJ_sVXyToxFHfgHDvafsNw!2e0!6shttps:%2F%2Fstreetviewpixels-pa.googleapis.com%2Fv1%2Fthumbnail%3Fcb_client%3Dmaps_sv.tactile%26w%3D900%26h%3D600%26pitch%3D-5.65189321189014%26panoid%3DrJ_sVXyToxFHfgHDvafsNw%26yaw%3D115.85355644268819!7i16384!8i8192!4m16!1m9!3m8!1s0x9584dea049a0f1e5:0x723a3a938bbc32eb!2sC%C3%B3rdoba+3068,+B7602CAF+Mar+del+Plata,+Provincia+de+Buenos+Aires,+Argentina!3b1!8m2!3d-38.0104545!4d-57.5556471!10e5!16s%2Fg%2F11f3w1nnm1!3m5!1s0x9584dea049afa063:0x3d327ea0788c0499!8m2!3d-38.0104238!4d-57.5556416!16s%2Fg%2F11bwf7fsp0?coh=205410&amp;entry=ttu&amp;g_ep=EgoyMDI0MTAwMi4xIKXMDSoASAFQAw%3D%3D</v>
+        <v>C.C Multicentro El Viñedo, Valencia</v>
       </c>
       <c r="F26" t="str">
-        <v>+54 911 5723-6341</v>
+        <v>https://www.google.com/maps/place/Multicentre+Vineyard/@10.2094622,-68.00859,16.25z/data=!4m6!3m5!1s0x8e805d9a4ddaf96b:0x6cd0bb2174ab91b7!8m2!3d10.2131461!4d-68.0093357!16s%2Fg%2F1hm4cgzwy?entry=ttu&amp;g_ep=EgoyMDI0MTAwMi4xIKXMDSoASAFQAw%3D%3D</v>
       </c>
       <c r="G26" t="str">
-        <v>ventas@32fouette.com.ar</v>
+        <v>+58 412-4330767</v>
       </c>
       <c r="H26" t="str">
-        <v/>
+        <v>volevenezuela@gmail.com</v>
       </c>
       <c r="I26" t="str">
-        <v/>
-      </c>
-      <c r="J26" t="str">
-        <v>https://fouette.com.ar/</v>
+        <v>https://www.instagram.com/vole.ve/</v>
       </c>
       <c r="K26" t="str">
-        <v>media-1336.jpg</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="str">
-        <v>FOUETTE</v>
-      </c>
-      <c r="B27" t="str">
-        <v>1250</v>
-      </c>
-      <c r="C27" t="str">
-        <v>argentina</v>
-      </c>
-      <c r="D27" t="str">
-        <v>Viamonte, 1177 (1053) – Cap. Fed.</v>
-      </c>
-      <c r="E27" t="str">
-        <v>https://www.google.com/maps/place/FOUETTE/@-34.6003997,-58.3835588,3a,75y,320.29h,91.59t/data=!3m6!1e1!3m4!1sjz1sTnmoBFKtHjZL204GUg!2e0!7i16384!8i8192!4m16!1m9!3m8!1s0x95bccac7d473326f:0xa54ea16bec298df1!2sViamonte+1177,+C1053ABW+Cdad.+Aut%C3%B3noma+de+Buenos+Aires,+Argentina!3b1!8m2!3d-34.6003047!4d-58.3835845!10e5!16s%2Fg%2F11c5c49hth!3m5!1s0x95bccac7d473326f:0x72f4b58c49784070!8m2!3d-34.6003114!4d-58.3835836!16s%2Fg%2F11b6jh29ll?coh=205409&amp;entry=ttu&amp;g_ep=EgoyMDI0MTAwMi4xIKXMDSoASAFQAw%3D%3D</v>
-      </c>
-      <c r="F27" t="str">
-        <v>+54 911 5723 7944</v>
-      </c>
-      <c r="G27" t="str">
-        <v>ventas@32fouette.com.ar</v>
-      </c>
-      <c r="H27" t="str">
-        <v/>
-      </c>
-      <c r="I27" t="str">
-        <v/>
-      </c>
-      <c r="J27" t="str">
-        <v>https://fouette.com.ar/</v>
-      </c>
-      <c r="K27" t="str">
-        <v>media-1335.jpg</v>
+        <v>https://treinta.shop/vol-a47b97</v>
+      </c>
+      <c r="L26" t="str">
+        <v>Punta-Carretas-3.jpg</v>
+      </c>
+      <c r="M26">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K27"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M26"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>